<commit_message>
changes in OTR dropdown
</commit_message>
<xml_diff>
--- a/vtsfrontend/public/images/DeactivationSample.xlsx
+++ b/vtsfrontend/public/images/DeactivationSample.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29409"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB4A2219-2500-447C-B3D1-BF5EB2F50D43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{159DDA47-4701-49C8-AB86-37103FA8022A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{F806F7BF-0198-46A7-83E9-A9F78B57442D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,6 +27,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -34,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>MILLER_TRANSPORTER_ID</t>
   </si>
@@ -69,6 +71,9 @@
     <t>OTR</t>
   </si>
   <si>
+    <t>otrMonth</t>
+  </si>
+  <si>
     <t>vehicle1</t>
   </si>
   <si>
@@ -78,6 +83,9 @@
     <t>vehicle3</t>
   </si>
   <si>
+    <t>DeactivationDate</t>
+  </si>
+  <si>
     <t>Employee_Name</t>
   </si>
   <si>
@@ -97,9 +105,6 @@
   </si>
   <si>
     <t>Remark3</t>
-  </si>
-  <si>
-    <t>DeactivationDate</t>
   </si>
   <si>
     <t>Deactivation_letterHead</t>
@@ -112,7 +117,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -523,22 +528,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F81F8347-5402-4F7C-B1C8-B9DD497780B6}">
-  <dimension ref="A1:W2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:X2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="38.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="29.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="24" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="38.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="41.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="38.28515625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="41.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -582,36 +588,39 @@
         <v>13</v>
       </c>
       <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="P1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="W1" s="3" t="s">
+      <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X1" s="3" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24">
       <c r="F2" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>